<commit_message>
Refatora catalogo para Excel e prepara integracoes Azure
</commit_message>
<xml_diff>
--- a/data/imports/materials.xlsx
+++ b/data/imports/materials.xlsx
@@ -502,7 +502,6 @@
           <t>Ordinário</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>incluir; ordinario; novo empenho</t>
@@ -513,7 +512,6 @@
           <t>Passo a passo para inclusão de um empenho do tipo ordinário.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>POP_101__empenho-inclusao-ordinario.docx</t>
@@ -549,7 +547,6 @@
           <t>Global</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>incluir; global</t>
@@ -560,7 +557,6 @@
           <t>Procedimento para gerar um empenho global com múltiplas parcelas.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>POP_102__empenho-inclusao-global.docx</t>
@@ -596,7 +592,6 @@
           <t>Estimativa</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>incluir; estimativa; serviços</t>
@@ -607,7 +602,6 @@
           <t>Como realizar a inclusão de um empenho por estimativa.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>POP_103__empenho-inclusao-estimativa.docx</t>
@@ -638,8 +632,6 @@
           <t>Conceitos</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>tipos; introdução; teoria</t>
@@ -655,7 +647,6 @@
           <t>https://youtube.com/watch?v=emp_vis_1</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -686,7 +677,6 @@
           <t>Reforço</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>reforçar; aumentar valor</t>
@@ -697,7 +687,6 @@
           <t>Instruções para realizar o reforço de saldo de um empenho existente.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>POP_105__empenho-reforco.docx</t>
@@ -748,7 +737,6 @@
           <t>Como anular totalmente o saldo de um empenho.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>POP_106__empenho-anulacao-total.docx</t>
@@ -799,7 +787,6 @@
           <t>Como realizar a anulação parcial (estorno parcial) do empenho.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>POP_107__empenho-anulacao-parcial.docx</t>
@@ -835,7 +822,6 @@
           <t>Anulação</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>vídeo; anulação; prática</t>
@@ -851,7 +837,6 @@
           <t>https://youtube.com/watch?v=emp_anula_2</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -882,7 +867,6 @@
           <t>Saldo</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>ver saldo; consulta; relatorio</t>
@@ -893,7 +877,6 @@
           <t>Passo a passo para consultar os saldos e o histórico de execuções do empenho.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>POP_109__empenho-consulta-saldo.docx</t>
@@ -929,7 +912,6 @@
           <t>Histórico</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>auditoria; historico; alteracoes</t>
@@ -940,7 +922,6 @@
           <t>Como verificar quem realizou alterações em um empenho específico.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>POP_110__empenho-historico.docx</t>
@@ -991,7 +972,6 @@
           <t>Procedimento para liquidar notas fiscais de material de consumo.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>POP_201__liq-material-consumo.docx</t>
@@ -1042,7 +1022,6 @@
           <t>Procedimento para liquidar notas fiscais de material permanente (bens).</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>POP_202__liq-material-permanente.docx</t>
@@ -1078,7 +1057,6 @@
           <t>Serviços</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>liquidar; serviços; terceiros</t>
@@ -1089,7 +1067,6 @@
           <t>Como realizar a liquidação de notas fiscais ou faturas de prestação de serviços.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>POP_203__liq-servicos.docx</t>
@@ -1125,7 +1102,6 @@
           <t>Fluxo</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>atesto; recebimento; teoria</t>
@@ -1141,7 +1117,6 @@
           <t>https://youtube.com/watch?v=liq_fluxo_1</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1172,7 +1147,6 @@
           <t>Folha</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>liquidar; folha; salarios</t>
@@ -1183,7 +1157,6 @@
           <t>Procedimentos específicos para inclusão da liquidação da folha de pagamento.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>POP_205__liq-folha.docx</t>
@@ -1219,7 +1192,6 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>estornar; cancelar; erro</t>
@@ -1230,7 +1202,6 @@
           <t>Passo a passo para estornar uma nota de liquidação lançada indevidamente.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>POP_206__liq-estorno-total.docx</t>
@@ -1266,7 +1237,6 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>estornar; ajuste; correção</t>
@@ -1277,7 +1247,6 @@
           <t>Como corrigir parcialmente valores de uma nota de liquidação via estorno.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>POP_207__liq-estorno-parcial.docx</t>
@@ -1313,7 +1282,6 @@
           <t>Exceções</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>erros; solução; ajuda; vídeo</t>
@@ -1329,7 +1297,6 @@
           <t>https://youtube.com/watch?v=liq_erros_2</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1360,7 +1327,6 @@
           <t>Adiantamento</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>suprimento; fundos; viagens</t>
@@ -1371,7 +1337,6 @@
           <t>Regras para liquidação de empenhos de suprimento de fundos/adiantamento.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>POP_209__liq-adiantamento.docx</t>
@@ -1407,7 +1372,6 @@
           <t>Notas</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>buscar; pesquisar; notas liquidação</t>
@@ -1418,7 +1382,6 @@
           <t>Como consultar a lista e a situação de notas de liquidação geradas.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>POP_210__liq-consulta-notas.docx</t>
@@ -1469,7 +1432,6 @@
           <t>Geração de Ordem Bancária para pagamento de fornecedores.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>POP_301__pag-ob-fornecedor.docx</t>
@@ -1505,7 +1467,6 @@
           <t>Inclusão</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>programar; pd; fluxo de caixa</t>
@@ -1516,7 +1477,6 @@
           <t>Como incluir a Programação de Desembolso antes do pagamento efetivo.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>POP_302__pag-pd.docx</t>
@@ -1552,7 +1512,6 @@
           <t>Fluxo</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>teoria; ordem; processo</t>
@@ -1568,7 +1527,6 @@
           <t>https://youtube.com/watch?v=pag_fluxo_1</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1599,7 +1557,6 @@
           <t>Tributos Federais</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>reter; imposto; irrf; inss</t>
@@ -1610,7 +1567,6 @@
           <t>Guia para registrar e destacar retenções tributárias no momento do pagamento.</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>POP_304__pag-retencoes-federais.docx</t>
@@ -1661,7 +1617,6 @@
           <t>Como destacar a retenção do Imposto Sobre Serviços (ISS).</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>POP_305__pag-retencoes-iss.docx</t>
@@ -1697,7 +1652,6 @@
           <t>OB</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>cancelar pagamento; estorno bancario</t>
@@ -1708,7 +1662,6 @@
           <t>Como registrar o cancelamento ou a devolução de uma Ordem Bancária rejeitada.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>POP_306__pag-cancelamento-ob.docx</t>
@@ -1744,7 +1697,6 @@
           <t>Folha</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>ob folha; salarios; servidores</t>
@@ -1755,7 +1707,6 @@
           <t>Rotina para a efetivação do pagamento em lote de servidores.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>POP_307__pag-ob-folha.docx</t>
@@ -1786,8 +1737,6 @@
           <t>Retorno Bancário</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>arquivo retorno; erro banco; vídeo</t>
@@ -1803,7 +1752,6 @@
           <t>https://youtube.com/watch?v=pag_retorno_2</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1834,7 +1782,6 @@
           <t>Situação</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>ver status; pago; pendente</t>
@@ -1845,7 +1792,6 @@
           <t>Como saber se o fornecedor já foi pago ou se está pendente.</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>POP_309__pag-consulta-situacao.docx</t>
@@ -1881,7 +1827,6 @@
           <t>Pendentes</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>relatorio; a pagar; divida</t>
@@ -1892,7 +1837,6 @@
           <t>Emissão do relatório de restos a pagar e empenhos liquidados não pagos.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>POP_310__pag-relatorio-pendentes.docx</t>
@@ -1943,7 +1887,6 @@
           <t>Como realizar a conciliação entre as contas do GRP e os extratos bancários.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>POP_401__cont-conciliacao.docx</t>
@@ -1979,7 +1922,6 @@
           <t>Manuais</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>partida dobrada; debito credito; diario</t>
@@ -1990,7 +1932,6 @@
           <t>Guia para realizar lançamentos contábeis típicos (débito/crédito) manuais.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>POP_402__cont-lancamentos.docx</t>
@@ -2026,7 +1967,6 @@
           <t>Plano de Contas</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>pcasp; teoria; contas; vídeo</t>
@@ -2042,7 +1982,6 @@
           <t>https://youtube.com/watch?v=cont_pcasp_1</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2073,7 +2012,6 @@
           <t>Encerramento</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>fechar ano; balanço; virada</t>
@@ -2084,7 +2022,6 @@
           <t>Procedimentos necessários para o fechamento do exercício fiscal no GRP.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>POP_404__cont-encerramento.docx</t>
@@ -2120,7 +2057,6 @@
           <t>Abertura</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>abrir ano; saldo inicial; janeiro</t>
@@ -2131,7 +2067,6 @@
           <t>Passos para iniciar a contabilidade em um novo ano civil.</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>POP_405__cont-abertura.docx</t>
@@ -2182,7 +2117,6 @@
           <t>Como extrair o relatório consolidado do Balanço Patrimonial.</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>POP_406__cont-balanco-patrimonial.docx</t>
@@ -2233,7 +2167,6 @@
           <t>Emissão da Demonstração das Variações Patrimoniais.</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>POP_407__cont-dve.docx</t>
@@ -2269,7 +2202,6 @@
           <t>Auditoria</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>auditar; inconsistencias; vídeo</t>
@@ -2285,7 +2217,6 @@
           <t>https://youtube.com/watch?v=cont_auditoria_2</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2331,7 +2262,6 @@
           <t>Como pesquisar o detalhamento do Razão Contábil de uma conta específica.</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>POP_409__cont-razao.docx</t>
@@ -2382,7 +2312,6 @@
           <t>Impressão e consulta do Livro Diário com toda a movimentação.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>POP_410__cont-diario.docx</t>

</xml_diff>